<commit_message>
atualização motor  coletor central com  selenum
</commit_message>
<xml_diff>
--- a/planilhacarros.xlsx
+++ b/planilhacarros.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
   <si>
     <t>id</t>
   </si>
@@ -34,19 +34,34 @@
     <t>dados_json</t>
   </si>
   <si>
-    <t>47f353d0766a6c86ada4cf9f518112887dba2fc73a81cb5edf3dc364f31146e5</t>
+    <t>479d135025c73ee0a00aff384888892b</t>
+  </si>
+  <si>
+    <t>cc67448e661b6f95ca1fbd6576d1d2cf</t>
   </si>
   <si>
     <t>a6824b700ae926300092e349462ee626ff490eb667f96d8caf7962078e8e82ca</t>
   </si>
   <si>
+    <t>cf46e5f06eeb13afcc04e9c86e009ccb</t>
+  </si>
+  <si>
     <t>25f57b18e092da55333453dbfbd2dab209ded9cb8fb6b4b77a7993ac28d22378</t>
   </si>
   <si>
+    <t>6073dad92eaf48ad5a3133baaed13b4d</t>
+  </si>
+  <si>
+    <t>be607e7cc4c8f47b49fda47b17f9477e</t>
+  </si>
+  <si>
     <t>RJ</t>
   </si>
   <si>
-    <t>eventual contratação de empresa especializada para prestar serviços de locação de veículos, blindados, van executiva e fretamento de ônibus com transporte municipal, intermunicipal e interestadual para atender a demanda do comando militar do leste e suas omds.</t>
+    <t>registro de preços para futura e eventual contratação de empresa especializada para prestação de serviços de locação de veículos automotores, sem condutor e sem fornecimento de combustível, para atender as necessidades da secretaria municipal de assistência social e cidadania – semasc, em conformidade com o edital e seus anexos.</t>
+  </si>
+  <si>
+    <t>contratação de empresa especializada para locação de veículos pelo sistema “on demand”</t>
   </si>
   <si>
     <t xml:space="preserve">registro de preços para prestação de serviço de locação de veículos, sem combustível, com e sem motorista, para atividades de operação de tráfego e apoio às unidades da mobi-rio, conforme as especificações constantes deste edital e/ou do termo de referência. </t>
@@ -55,13 +70,22 @@
     <t>o presente tem por objeto a contratação de empresa especializada na locação de veículos automotores de passeio e utilitários, sem condutor e com quilometragem livre, para atender às necessidades operacionais, de fiscalização turística e de representação institucional da niterói empresa de lazer e turismo s/a – neltur.</t>
   </si>
   <si>
-    <t>{'srp': True, 'processo': '64283.024331 /202', 'anoCompra': 2025, 'amparoLegal': {'nome': 'Lei 14.133/2021, Art. 28, I', 'codigo': 1, 'descricao': 'pregão: modalidade de licitação obrigatória para aquisição de bens e serviços comuns'}, 'usuarioNome': 'Compras.gov.br', 'dataInclusao': '2026-05-05T07:11:42', 'modalidadeId': 6, 'numeroCompra': '90014', 'objetoCompra': 'Eventual contratação de empresa especializada para prestar serviços de Locação de Veículos, Blindados, Van Executiva e Fretamento de Ônibus com transporte municipal, intermunicipal e interestadual para atender a demanda do Comando Militar do Leste e suas OMDS.', 'unidadeOrgao': {'ufNome': 'Rio de Janeiro', 'ufSigla': 'RJ', 'codigoIbge': '3304557', 'nomeUnidade': 'COMANDO DO COMANDO MILITAR DO LESTE/RJ', 'codigoUnidade': '160299', 'municipioNome': 'Rio de Janeiro'}, 'modoDisputaId': 1, 'orgaoEntidade': {'cnpj': '00394452000103', 'poderId': 'E', 'esferaId': 'F', 'razaoSocial': 'COMANDO DO EXERCITO'}, 'modalidadeNome': 'Pregão - Eletrônico', 'orgaoSubRogado': None, 'dataAtualizacao': '2026-05-05T07:11:42', 'modoDisputaNome': 'Aberto', 'sequencialCompra': 25482, 'situacaoCompraId': 1, 'unidadeSubRogada': None, 'emendaParlamentar': None, 'linkSistemaOrigem': 'https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=acompanhamento-compra&amp;compra=16029905900142025', 'dataPublicacaoPncp': '2026-05-05T07:11:42', 'numeroControlePNCP': '00394452000103-1-025482/2025', 'situacaoCompraNome': 'Divulgada no PNCP', 'valorTotalEstimado': 7864193.3, 'fontesOrcamentarias': [], 'dataAberturaProposta': '2026-05-05T09:00:00', 'valorTotalHomologado': None, 'dataAtualizacaoGlobal': '2026-05-05T07:11:42', 'informacaoComplementar': 'Eventual contratação de empresa especializada para prestar serviços de Locação de Veículos, Blindados, Van Executiva e Fretamento de Ônibus com transporte municipal, intermunicipal e interestadual para atender a demanda do Comando Militar do Leste e suas OMDS. Para as respostas de esclarecimentos e impugnações deste edital acesse o link: https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=quadro-informativo&amp;compra=16029905900142025', 'linkProcessoEletronico': None, 'justificativaPresencial': None, 'dataEncerramentoProposta': '2026-05-26T09:00:00', 'tipoInstrumentoConvocatorioNome': 'Edital', 'tipoInstrumentoConvocatorioCodigo': 1}</t>
+    <t>registro de preço para locação de veículos automotores a pedido da secretaria municipal de saúde do município de bom jesus do itabapoana-rj.</t>
+  </si>
+  <si>
+    <t>{'srp': True, 'processo': '56/0114/2025 ', 'anoCompra': 2026, 'amparoLegal': {'nome': 'Lei 14.133/2021, Art. 28, I', 'codigo': 1, 'descricao': 'pregão: modalidade de licitação obrigatória para aquisição de bens e serviços comuns'}, 'usuarioNome': 'Compras.gov.br', 'dataInclusao': '2026-05-05T07:07:51', 'modalidadeId': 6, 'numeroCompra': '90007', 'objetoCompra': 'Registro de preços para futura e eventual CONTRATAÇÃO DE EMPRESA ESPECIALIZADA PARA PRESTAÇÃO DE SERVIÇOS DE LOCAÇÃO DE VEÍCULOS AUTOMOTORES, SEM CONDUTOR E SEM FORNECIMENTO DE COMBUSTÍVEL, para atender as necessidades da Secretaria Municipal de Assistência Social e Cidadania – SEMASC, em conformidade com o Edital e seus anexos.', 'unidadeOrgao': {'ufNome': 'Rio de Janeiro', 'ufSigla': 'RJ', 'codigoIbge': '3300456', 'nomeUnidade': 'MRJ-PREFEITURA MUNICIPAL DE BELFORD ROXO', 'codigoUnidade': '982909', 'municipioNome': 'Belford Roxo'}, 'modoDisputaId': 1, 'orgaoEntidade': {'cnpj': '39485438000142', 'poderId': 'N', 'esferaId': 'M', 'razaoSocial': 'MUNICIPIO DE BELFORD ROXO'}, 'modalidadeNome': 'Pregão - Eletrônico', 'orgaoSubRogado': None, 'dataAtualizacao': '2026-05-21T07:36:57', 'modoDisputaNome': 'Aberto', 'sequencialCompra': 23, 'situacaoCompraId': 1, 'unidadeSubRogada': None, 'emendaParlamentar': None, 'linkSistemaOrigem': 'https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=acompanhamento-compra&amp;compra=98290905900072026', 'dataPublicacaoPncp': '2026-05-05T07:07:51', 'numeroControlePNCP': '39485438000142-1-000023/2026', 'situacaoCompraNome': 'Divulgada no PNCP', 'valorTotalEstimado': 3483050.76, 'fontesOrcamentarias': [], 'dataAberturaProposta': '2026-05-21T09:00:00', 'valorTotalHomologado': None, 'dataAtualizacaoGlobal': '2026-05-21T07:36:58', 'informacaoComplementar': 'Em caso de divergência entre o descritivo do sistema e do edital este último prevalecerá Para as respostas de esclarecimentos e impugnações deste edital acesse o link: https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=quadro-informativo&amp;compra=98290905900072026', 'linkProcessoEletronico': None, 'justificativaPresencial': None, 'dataEncerramentoProposta': '2026-06-10T10:00:00', 'tipoInstrumentoConvocatorioNome': 'Edital', 'tipoInstrumentoConvocatorioCodigo': 1}</t>
+  </si>
+  <si>
+    <t>{'srp': False, 'processo': '00002870/2026', 'anoCompra': 2026, 'amparoLegal': {'nome': 'Lei 14.133/2021, Art. 28, I', 'codigo': 1, 'descricao': 'pregão: modalidade de licitação obrigatória para aquisição de bens e serviços comuns'}, 'usuarioNome': 'Compras.gov.br', 'dataInclusao': '2026-05-19T07:10:38', 'modalidadeId': 6, 'numeroCompra': '90004', 'objetoCompra': 'Contratação de Empresa Especializada para Locação de Veículos pelo Sistema “On Demand”', 'unidadeOrgao': {'ufNome': 'Rio de Janeiro', 'ufSigla': 'RJ', 'codigoIbge': '3306305', 'nomeUnidade': 'EMP DE PROC. DE DADOS DE VOLTA REDONDA - RJ', 'codigoUnidade': '926754', 'municipioNome': 'Volta Redonda'}, 'modoDisputaId': 3, 'orgaoEntidade': {'cnpj': '32512501000143', 'poderId': 'N', 'esferaId': 'M', 'razaoSocial': 'MUNICIPIO DE VOLTA REDONDA'}, 'modalidadeNome': 'Pregão - Eletrônico', 'orgaoSubRogado': None, 'dataAtualizacao': '2026-05-19T07:10:38', 'modoDisputaNome': 'Aberto-Fechado', 'sequencialCompra': 177, 'situacaoCompraId': 1, 'unidadeSubRogada': None, 'emendaParlamentar': None, 'linkSistemaOrigem': 'https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=acompanhamento-compra&amp;compra=92675405900042026', 'dataPublicacaoPncp': '2026-05-19T07:10:38', 'numeroControlePNCP': '32512501000143-1-000177/2026', 'situacaoCompraNome': 'Divulgada no PNCP', 'valorTotalEstimado': 0.0, 'fontesOrcamentarias': [], 'dataAberturaProposta': '2026-05-19T08:00:00', 'valorTotalHomologado': None, 'dataAtualizacaoGlobal': '2026-05-19T07:10:38', 'informacaoComplementar': 'Se atentar as especificações contidas no Edital Para as respostas de esclarecimentos e impugnações deste edital acesse o link: https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=quadro-informativo&amp;compra=92675405900042026', 'linkProcessoEletronico': None, 'justificativaPresencial': None, 'dataEncerramentoProposta': '2026-06-11T09:00:00', 'tipoInstrumentoConvocatorioNome': 'Edital', 'tipoInstrumentoConvocatorioCodigo': 1}</t>
   </si>
   <si>
     <t>{'srp': True, 'processo': '07300000746202625', 'anoCompra': 2026, 'amparoLegal': {'nome': 'Lei 14.133/2021, Art. 28, I', 'codigo': 1, 'descricao': 'pregão: modalidade de licitação obrigatória para aquisição de bens e serviços comuns'}, 'usuarioNome': 'Compras.gov.br', 'dataInclusao': '2026-05-15T07:10:28', 'modalidadeId': 6, 'numeroCompra': '90316', 'objetoCompra': 'Registro de preços para prestação de serviço de locação de veículos, sem combustível, com e sem motorista, para atividades de operação de tráfego e apoio às unidades da MOBI-RIO, conforme as especificações constantes deste Edital e/ou do Termo de Referência. ', 'unidadeOrgao': {'ufNome': 'Rio de Janeiro', 'ufSigla': 'RJ', 'codigoIbge': '3304557', 'nomeUnidade': 'PREFEITURA MUNICIPAL DO RIO DE JANEIRO - RJ', 'codigoUnidade': '986001', 'municipioNome': 'Rio de Janeiro'}, 'modoDisputaId': 3, 'orgaoEntidade': {'cnpj': '42498733000148', 'poderId': 'N', 'esferaId': 'M', 'razaoSocial': 'MUNICIPIO DE RIO DE JANEIRO'}, 'modalidadeNome': 'Pregão - Eletrônico', 'orgaoSubRogado': None, 'dataAtualizacao': '2026-05-15T07:10:28', 'modoDisputaNome': 'Aberto-Fechado', 'sequencialCompra': 952, 'situacaoCompraId': 1, 'unidadeSubRogada': None, 'emendaParlamentar': None, 'linkSistemaOrigem': 'https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=acompanhamento-compra&amp;compra=98600105903162026', 'dataPublicacaoPncp': '2026-05-15T07:10:28', 'numeroControlePNCP': '42498733000148-1-000952/2026', 'situacaoCompraNome': 'Divulgada no PNCP', 'valorTotalEstimado': 0.0, 'fontesOrcamentarias': [], 'dataAberturaProposta': '2026-05-15T08:00:00', 'valorTotalHomologado': None, 'dataAtualizacaoGlobal': '2026-05-15T07:10:29', 'informacaoComplementar': ' Para as respostas de esclarecimentos e impugnações deste edital acesse o link: https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=quadro-informativo&amp;compra=98600105903162026', 'linkProcessoEletronico': None, 'justificativaPresencial': None, 'dataEncerramentoProposta': '2026-05-29T11:00:00', 'tipoInstrumentoConvocatorioNome': 'Edital', 'tipoInstrumentoConvocatorioCodigo': 1}</t>
   </si>
   <si>
     <t>{'srp': False, 'processo': '9900021427/2026', 'anoCompra': 2026, 'amparoLegal': {'nome': 'Lei 14.133/2021, Art. 28, I', 'codigo': 1, 'descricao': 'pregão: modalidade de licitação obrigatória para aquisição de bens e serviços comuns'}, 'usuarioNome': 'Compras.gov.br', 'dataInclusao': '2026-05-18T07:08:33', 'modalidadeId': 6, 'numeroCompra': '90002', 'objetoCompra': 'O presente tem por objeto a contratação de empresa especializada na locação de veículos automotores de passeio e utilitários, sem condutor e com quilometragem livre, para atender às necessidades operacionais, de fiscalização turística e de representação institucional da Niterói Empresa de Lazer e Turismo S/A – NELTUR.', 'unidadeOrgao': {'ufNome': 'Rio de Janeiro', 'ufSigla': 'RJ', 'codigoIbge': '3303302', 'nomeUnidade': 'NITERÓI EMPRESA DE LAZER E TURISMO S/A - RJ', 'codigoUnidade': '929395', 'municipioNome': 'Niterói'}, 'modoDisputaId': 1, 'orgaoEntidade': {'cnpj': '29541968000107', 'poderId': 'N', 'esferaId': 'N', 'razaoSocial': 'NITEROI - EMPRESA DE LAZER E TURISMO S/A - NELTUR'}, 'modalidadeNome': 'Pregão - Eletrônico', 'orgaoSubRogado': None, 'dataAtualizacao': '2026-05-18T07:08:33', 'modoDisputaNome': 'Aberto', 'sequencialCompra': 2, 'situacaoCompraId': 1, 'unidadeSubRogada': None, 'emendaParlamentar': None, 'linkSistemaOrigem': 'https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=acompanhamento-compra&amp;compra=92939505900022026', 'dataPublicacaoPncp': '2026-05-18T07:08:33', 'numeroControlePNCP': '29541968000107-1-000002/2026', 'situacaoCompraNome': 'Divulgada no PNCP', 'valorTotalEstimado': 0.0, 'fontesOrcamentarias': [], 'dataAberturaProposta': '2026-05-18T09:00:00', 'valorTotalHomologado': None, 'dataAtualizacaoGlobal': '2026-05-18T07:08:33', 'informacaoComplementar': ' Para as respostas de esclarecimentos e impugnações deste edital acesse o link: https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=quadro-informativo&amp;compra=92939505900022026', 'linkProcessoEletronico': None, 'justificativaPresencial': None, 'dataEncerramentoProposta': '2026-06-01T10:00:00', 'tipoInstrumentoConvocatorioNome': 'Edital', 'tipoInstrumentoConvocatorioCodigo': 1}</t>
+  </si>
+  <si>
+    <t>{'srp': True, 'processo': '030208/000581/26', 'anoCompra': 2026, 'amparoLegal': {'nome': 'Lei 14.133/2021, Art. 28, I', 'codigo': 1, 'descricao': 'pregão: modalidade de licitação obrigatória para aquisição de bens e serviços comuns'}, 'usuarioNome': 'Compras.gov.br', 'dataInclusao': '2026-05-22T07:42:31', 'modalidadeId': 6, 'numeroCompra': '90023', 'objetoCompra': 'Registro de preço para locação de veículos automotores a pedido da Secretaria Municipal de Saúde do Município de Bom Jesus do Itabapoana-RJ.', 'unidadeOrgao': {'ufNome': 'Rio de Janeiro', 'ufSigla': 'RJ', 'codigoIbge': '3300605', 'nomeUnidade': 'PREFEITURA MUNICIPAL BOM JESUS DO ITABAPOANA', 'codigoUnidade': '985811', 'municipioNome': 'Bom Jesus do Itabapoana'}, 'modoDisputaId': 1, 'orgaoEntidade': {'cnpj': '29112760000172', 'poderId': 'E', 'esferaId': 'M', 'razaoSocial': 'BOM JESUS DO ITABAPOANA PREFEITURA'}, 'modalidadeNome': 'Pregão - Eletrônico', 'orgaoSubRogado': None, 'dataAtualizacao': '2026-05-22T07:42:31', 'modoDisputaNome': 'Aberto', 'sequencialCompra': 167, 'situacaoCompraId': 1, 'unidadeSubRogada': None, 'emendaParlamentar': None, 'linkSistemaOrigem': 'https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=acompanhamento-compra&amp;compra=98581105900232026', 'dataPublicacaoPncp': '2026-05-22T07:42:31', 'numeroControlePNCP': '29112760000172-1-000167/2026', 'situacaoCompraNome': 'Divulgada no PNCP', 'valorTotalEstimado': 654569.7, 'fontesOrcamentarias': [], 'dataAberturaProposta': '2026-05-22T08:00:00', 'valorTotalHomologado': None, 'dataAtualizacaoGlobal': '2026-05-22T07:42:31', 'informacaoComplementar': ' Para as respostas de esclarecimentos e impugnações deste edital acesse o link: https://cnetmobile.estaleiro.serpro.gov.br/comprasnet-web/public/landing?destino=quadro-informativo&amp;compra=98581105900232026', 'linkProcessoEletronico': None, 'justificativaPresencial': None, 'dataEncerramentoProposta': '2026-06-08T09:00:00', 'tipoInstrumentoConvocatorioNome': 'Edital', 'tipoInstrumentoConvocatorioCodigo': 1}</t>
   </si>
 </sst>
 </file>
@@ -423,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -448,62 +472,142 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2">
-        <v>275351</v>
+        <v>306079</v>
       </c>
       <c r="B2" s="2">
-        <v>46162.60237744559</v>
+        <v>46169.07520127673</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3">
-        <v>288132</v>
+        <v>315565</v>
       </c>
       <c r="B3" s="2">
-        <v>46162.70168875143</v>
+        <v>46169.08276617506</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4">
-        <v>291610</v>
+        <v>288132</v>
       </c>
       <c r="B4" s="2">
-        <v>46162.72598467913</v>
+        <v>46162.70168875143</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
       </c>
       <c r="D4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>311791</v>
+      </c>
+      <c r="B5" s="2">
+        <v>46169.07738703379</v>
+      </c>
+      <c r="C5" t="s">
         <v>9</v>
       </c>
-      <c r="E4" t="s">
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>291610</v>
+      </c>
+      <c r="B6" s="2">
+        <v>46162.72598467913</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>313599</v>
+      </c>
+      <c r="B7" s="2">
+        <v>46169.08046262934</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8">
+        <v>321875</v>
+      </c>
+      <c r="B8" s="2">
+        <v>46169.08568111081</v>
+      </c>
+      <c r="C8" t="s">
         <v>12</v>
       </c>
-      <c r="F4" t="s">
-        <v>15</v>
+      <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>